<commit_message>
test: keep additional court samples
</commit_message>
<xml_diff>
--- a/court-search/sample_input.xlsx
+++ b/court-search/sample_input.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C2"/>
+  <dimension ref="A1:C7"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -450,6 +450,91 @@
         </is>
       </c>
     </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>인천지방법원</t>
+        </is>
+      </c>
+      <c r="B3" t="inlineStr">
+        <is>
+          <t>2026타인50938</t>
+        </is>
+      </c>
+      <c r="C3" t="inlineStr">
+        <is>
+          <t>주택</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>서울남부지방법원</t>
+        </is>
+      </c>
+      <c r="B4" t="inlineStr">
+        <is>
+          <t>2026타인3273</t>
+        </is>
+      </c>
+      <c r="C4" t="inlineStr">
+        <is>
+          <t>주택</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>서울남부지방법원</t>
+        </is>
+      </c>
+      <c r="B5" t="inlineStr">
+        <is>
+          <t>2026타인3274</t>
+        </is>
+      </c>
+      <c r="C5" t="inlineStr">
+        <is>
+          <t>주택</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>서울중앙지방법원</t>
+        </is>
+      </c>
+      <c r="B6" t="inlineStr">
+        <is>
+          <t>2026타인10046</t>
+        </is>
+      </c>
+      <c r="C6" t="inlineStr">
+        <is>
+          <t>주택</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>인천지방법원 부천지원</t>
+        </is>
+      </c>
+      <c r="B7" t="inlineStr">
+        <is>
+          <t>2026타인10353</t>
+        </is>
+      </c>
+      <c r="C7" t="inlineStr">
+        <is>
+          <t>주택</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>